<commit_message>
Apply review decisions to India infusion pump matrix
Peach for distributor listings, Spaceplus Perfusor removed (not offered
in India), Agilia VP MC WiFi pending distributor check, official revenue
only on slide, USD at latest ECB rate (1.1204, 5-Oct-2026).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014jxHyvpwsKVbJ3RxrkkV1k
</commit_message>
<xml_diff>
--- a/Infusion_Pumps_India/Infusion_Pump_Classification_India.xlsx
+++ b/Infusion_Pumps_India/Infusion_Pump_Classification_India.xlsx
@@ -104,7 +104,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF59D"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -236,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -262,7 +262,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -270,7 +270,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -283,16 +283,19 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -814,10 +817,9 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>EUR 9.40B FY25 group sales (~USD 10.79B*)
-Hospital Care div.: EUR 5.09B
-India entity FY25: INR 500-750 Cr
-(see Revenue tab)</t>
+          <t>EUR 9.40B FY25 group sales (~USD 10.53B*)
+of which Hospital Care div. (incl. infusion therapy): EUR 5.09B
+Source: B. Braun Annual Report 2025</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
@@ -830,11 +832,7 @@
           <t>Perfusor compactplus**</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
-        <is>
-          <t>Spaceplus Perfusor (not verified in India)</t>
-        </is>
-      </c>
+      <c r="F6" s="15" t="n"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>Infusomat fmS</t>
@@ -854,7 +852,7 @@
         <is>
           <t>- Standard columns were blank: add Perfusor compact, compact S, Infusomat fmS, Infusomat P
 - compactplus &amp; Space pumps -&gt; Smart** (connectivity is optional)
-- 'Perfusor Space Plus' NOT on India catalogue -&gt; remove/footnote
+- 'Perfusor Space Plus' removed: not offered in India (catalogue + distributors)
 - 'Infusomat Space' -&gt; India lists Infusomat Space P
 - 'Infusomat Space Place' typo -&gt; Spaceplus Infusomat
 - Add Infusomat compactplus P</t>
@@ -863,7 +861,7 @@
       <c r="K6" s="16" t="n"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Not verified in India - needs manual check / remove</t>
+          <t>Pending confirmation of an Indian distributor listing</t>
         </is>
       </c>
     </row>
@@ -881,7 +879,7 @@
           <t>Perfusor Space**</t>
         </is>
       </c>
-      <c r="F7" s="18" t="n"/>
+      <c r="F7" s="17" t="n"/>
       <c r="G7" s="14" t="inlineStr">
         <is>
           <t>Infusomat P</t>
@@ -901,7 +899,7 @@
       <c r="C8" s="10" t="n"/>
       <c r="D8" s="18" t="n"/>
       <c r="E8" s="18" t="n"/>
-      <c r="F8" s="18" t="n"/>
+      <c r="F8" s="10" t="n"/>
       <c r="G8" s="18" t="n"/>
       <c r="H8" s="14" t="inlineStr">
         <is>
@@ -924,13 +922,12 @@
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>EUR 8.61B FY25 Kabi revenue (~USD 9.89B*)
-MedTech: EUR 1.61B
-India entity FY25: INR 750-1,000 Cr
-(see Revenue tab)</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="n"/>
+          <t>EUR 8.61B FY25 Kabi revenue (~USD 9.65B*)
+of which MedTech (incl. infusion pumps): EUR 1.61B
+Source: Fresenius Annual Report 2025</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="n"/>
       <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Infusia SP7s (SP7sED3)</t>
@@ -941,22 +938,22 @@
           <t>Agilia SP MC WiFi</t>
         </is>
       </c>
-      <c r="G9" s="19" t="n"/>
+      <c r="G9" s="15" t="n"/>
       <c r="H9" s="14" t="inlineStr">
         <is>
           <t>Infusia VP7s (VP7sED3)</t>
         </is>
       </c>
-      <c r="I9" s="15" t="inlineStr">
-        <is>
-          <t>Agilia VP MC WiFi (not verified in India)</t>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>Agilia VP MC WiFi (pending India confirmation)</t>
         </is>
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
           <t>- Add Agilia SP (Smart), Agilia SP MC &amp; SP TIVA (Smart**)
-- Agilia VP (distributor only) -&gt; Volumetric Smart, yellow
-- Agilia VP MC WiFi: no India listing found -&gt; verify or remove
+- Agilia VP (distributor only) -&gt; Volumetric Smart, peach
+- Agilia VP MC WiFi: pending distributor confirmation (keep only if an Indian listing is found)
 - Infusia SP7s/VP7s &amp; Agilia SP MC WiFi confirmed</t>
         </is>
       </c>
@@ -1016,7 +1013,7 @@
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>** Smart** = drug library + connectivity optional (separately sold data module / WiFi variant).  * USD at EUR/USD 1.148, the rate implied by the sample slide - confirm FX basis (see Revenue tab).</t>
+          <t>** Smart** = drug library + connectivity optional (separately sold data module / WiFi variant).  * USD converted at ECB EUR/USD reference rate 1.1204 (5-Oct-2026), latest available; sample slide had used ~1.148.</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1025,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="J9:J12"/>
     <mergeCell ref="D9:D12"/>
     <mergeCell ref="C9:C12"/>
@@ -1043,6 +1040,7 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="B6:B8"/>
+    <mergeCell ref="F6:F8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1431,12 +1429,12 @@
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Connected (global only)</t>
+          <t>Excluded - not offered in India</t>
         </is>
       </c>
       <c r="G6" s="24" t="inlineStr">
         <is>
-          <t>Not verified in India</t>
+          <t>Not offered in India</t>
         </is>
       </c>
       <c r="H6" s="25" t="inlineStr">
@@ -1456,7 +1454,7 @@
       </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>REMOVE from India matrix (not listed on India catalogue) or footnote as global-only</t>
+          <t>REMOVED - not on B. Braun India catalogue; not found on Indian distributor sites (confirmed by project team, manual check)</t>
         </is>
       </c>
       <c r="L6" s="13" t="inlineStr">
@@ -2299,7 +2297,7 @@
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>ADD to Volumetric-Smart (yellow - distributor only)</t>
+          <t>ADD to Volumetric-Smart (peach - distributor only)</t>
         </is>
       </c>
       <c r="L19" s="13" t="inlineStr">
@@ -2319,7 +2317,7 @@
           <t>Fresenius Kabi</t>
         </is>
       </c>
-      <c r="B20" s="24" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>Agilia VP MC WiFi</t>
         </is>
@@ -2344,14 +2342,14 @@
           <t>Connected (global only)</t>
         </is>
       </c>
-      <c r="G20" s="24" t="inlineStr">
+      <c r="G20" s="28" t="inlineStr">
         <is>
           <t>Not verified in India</t>
         </is>
       </c>
-      <c r="H20" s="24" t="inlineStr">
-        <is>
-          <t>None found - not on FK India site or Arraymed</t>
+      <c r="H20" s="28" t="inlineStr">
+        <is>
+          <t>Pending - not on FK India site or Arraymed; IndiaMart search for team check: https://dir.indiamart.com/search.mp?ss=agilia+vp+mc+wifi</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
@@ -2366,7 +2364,7 @@
       </c>
       <c r="K20" s="13" t="inlineStr">
         <is>
-          <t>UNVERIFIED - provide the IndiaMart/distributor link, or remove</t>
+          <t>PENDING team confirmation of IndiaMart/distributor listing; remove if none</t>
         </is>
       </c>
       <c r="L20" s="13" t="inlineStr">
@@ -2429,7 +2427,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Revenue cross-check (FY2025)</t>
         </is>
@@ -2441,12 +2439,12 @@
           <t>EUR/USD rate (input)</t>
         </is>
       </c>
-      <c r="B2" s="29" t="n">
-        <v>1.148</v>
+      <c r="B2" s="30" t="n">
+        <v>1.1204</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Assumption: rate implied by sample slide (USD 10.79B / EUR 9.396B = USD 9.89B / EUR 8.612B = 1.148). Confirm whether average or closing rate is intended and replace.</t>
+          <t>ECB euro reference rate, latest available (5-Oct-2026): https://data.ecb.europa.eu/data/datasets/EXR/EXR.D.USD.EUR.SP00.A  |  For reference: 2025 annual average 1.1300; the sample slide implied ~1.148.</t>
         </is>
       </c>
     </row>
@@ -2523,10 +2521,10 @@
           <t>FY2025 (Dec-25)</t>
         </is>
       </c>
-      <c r="D5" s="30" t="n">
+      <c r="D5" s="31" t="n">
         <v>9396</v>
       </c>
-      <c r="E5" s="31">
+      <c r="E5" s="32">
         <f>IF(D5="","n/a",D5*$B$2/1000)</f>
         <v/>
       </c>
@@ -2537,7 +2535,7 @@
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>Matches (EUR 9,396mn x 1.148)</t>
+          <t>EUR figure matches; sample USD used ~1.148 -&gt; now USD 10.53B at latest ECB rate</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
@@ -2572,10 +2570,10 @@
           <t>FY2025</t>
         </is>
       </c>
-      <c r="D6" s="30" t="n">
+      <c r="D6" s="31" t="n">
         <v>5090.8</v>
       </c>
-      <c r="E6" s="31">
+      <c r="E6" s="32">
         <f>IF(D6="","n/a",D6*$B$2/1000)</f>
         <v/>
       </c>
@@ -2621,8 +2619,8 @@
           <t>FY2025 (Mar-25)</t>
         </is>
       </c>
-      <c r="D7" s="30" t="n"/>
-      <c r="E7" s="31">
+      <c r="D7" s="31" t="n"/>
+      <c r="E7" s="32">
         <f>IF(D7="","n/a",D7*$B$2/1000)</f>
         <v/>
       </c>
@@ -2633,7 +2631,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>Not on sample</t>
+          <t>UNOFFICIAL - not used on slide</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
@@ -2668,10 +2666,10 @@
           <t>FY2025 (Dec-25)</t>
         </is>
       </c>
-      <c r="D8" s="30" t="n">
+      <c r="D8" s="31" t="n">
         <v>8612</v>
       </c>
-      <c r="E8" s="31">
+      <c r="E8" s="32">
         <f>IF(D8="","n/a",D8*$B$2/1000)</f>
         <v/>
       </c>
@@ -2682,7 +2680,7 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>Matches (EUR 8,612mn x 1.148)</t>
+          <t>EUR figure matches; sample USD used ~1.148 -&gt; now USD 9.65B at latest ECB rate</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
@@ -2717,10 +2715,10 @@
           <t>FY2025</t>
         </is>
       </c>
-      <c r="D9" s="30" t="n">
+      <c r="D9" s="31" t="n">
         <v>1610</v>
       </c>
-      <c r="E9" s="31">
+      <c r="E9" s="32">
         <f>IF(D9="","n/a",D9*$B$2/1000)</f>
         <v/>
       </c>
@@ -2766,8 +2764,8 @@
           <t>FY2025 (Mar-25)</t>
         </is>
       </c>
-      <c r="D10" s="30" t="n"/>
-      <c r="E10" s="31">
+      <c r="D10" s="31" t="n"/>
+      <c r="E10" s="32">
         <f>IF(D10="","n/a",D10*$B$2/1000)</f>
         <v/>
       </c>
@@ -2778,7 +2776,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Not on sample</t>
+          <t>UNOFFICIAL - not used on slide</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
@@ -2870,7 +2868,7 @@
           <t>India catalogue - automated infusion systems (master list)</t>
         </is>
       </c>
-      <c r="C2" s="32" t="inlineStr">
+      <c r="C2" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/c/PRODUCTS0000000529/automated-infusion-systems</t>
         </is>
@@ -2902,7 +2900,7 @@
           <t>Perfusor compact</t>
         </is>
       </c>
-      <c r="C3" s="32" t="inlineStr">
+      <c r="C3" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000461</t>
         </is>
@@ -2934,7 +2932,7 @@
           <t>Perfusor compact S</t>
         </is>
       </c>
-      <c r="C4" s="32" t="inlineStr">
+      <c r="C4" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000145</t>
         </is>
@@ -2966,7 +2964,7 @@
           <t>Perfusor compactplus</t>
         </is>
       </c>
-      <c r="C5" s="32" t="inlineStr">
+      <c r="C5" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00010216</t>
         </is>
@@ -2998,7 +2996,7 @@
           <t>Data module compactplus (connectivity add-on)</t>
         </is>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00011150</t>
         </is>
@@ -3030,7 +3028,7 @@
           <t>compactplus brochure (p.5 data module, p.6 DoseGuard)</t>
         </is>
       </c>
-      <c r="C7" s="32" t="inlineStr">
+      <c r="C7" s="33" t="inlineStr">
         <is>
           <t>https://ecatalog.bbraun.com/eDoc/QlBSMDAwMDAwMDAwMDAwMDAwMTAwMDE4NTA5OTAwMDAw?openInline=true</t>
         </is>
@@ -3058,7 +3056,7 @@
           <t>Perfusor Space</t>
         </is>
       </c>
-      <c r="C8" s="32" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00001226</t>
         </is>
@@ -3090,7 +3088,7 @@
           <t>Infusomat fmS</t>
         </is>
       </c>
-      <c r="C9" s="32" t="inlineStr">
+      <c r="C9" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000618</t>
         </is>
@@ -3122,7 +3120,7 @@
           <t>Infusomat P</t>
         </is>
       </c>
-      <c r="C10" s="32" t="inlineStr">
+      <c r="C10" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000689</t>
         </is>
@@ -3154,7 +3152,7 @@
           <t>Infusomat compactplus</t>
         </is>
       </c>
-      <c r="C11" s="32" t="inlineStr">
+      <c r="C11" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00011042</t>
         </is>
@@ -3186,7 +3184,7 @@
           <t>Infusomat compactplus P</t>
         </is>
       </c>
-      <c r="C12" s="32" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00012086</t>
         </is>
@@ -3214,7 +3212,7 @@
           <t>Infusomat Space P</t>
         </is>
       </c>
-      <c r="C13" s="32" t="inlineStr">
+      <c r="C13" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00001230</t>
         </is>
@@ -3242,7 +3240,7 @@
           <t>Spaceplus Infusomat</t>
         </is>
       </c>
-      <c r="C14" s="32" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00011860</t>
         </is>
@@ -3274,7 +3272,7 @@
           <t>Annual Report 2025 (revenue)</t>
         </is>
       </c>
-      <c r="C15" s="32" t="inlineStr">
+      <c r="C15" s="33" t="inlineStr">
         <is>
           <t>https://www.bbraun.com/en/about-us/company/facts-and-figures/annual-report.html</t>
         </is>
@@ -3306,7 +3304,7 @@
           <t>Annual Report 2025 PDF (p.8, p.43)</t>
         </is>
       </c>
-      <c r="C16" s="32" t="inlineStr">
+      <c r="C16" s="33" t="inlineStr">
         <is>
           <t>https://www.bbraun.com/content/dam/b-braun/master/website-6/en/04_about-us/0401_company/facts-and-figures/2025_B_Braun_Annual_Report.pdf</t>
         </is>
@@ -3338,7 +3336,7 @@
           <t>India entity financials</t>
         </is>
       </c>
-      <c r="C17" s="32" t="inlineStr">
+      <c r="C17" s="33" t="inlineStr">
         <is>
           <t>https://www.tofler.in/b-braun-medical-india-private-limited/company/U33112MH1984PTC214514</t>
         </is>
@@ -3370,7 +3368,7 @@
           <t>compactplus system (global page)</t>
         </is>
       </c>
-      <c r="C18" s="32" t="inlineStr">
+      <c r="C18" s="33" t="inlineStr">
         <is>
           <t>https://www.bbraun.com/en/products-and-solutions/therapies/infusion-therapy/automated-infusion-systems/compactplus-system.html</t>
         </is>
@@ -3380,7 +3378,7 @@
           <t>Global website</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="28" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -3402,7 +3400,7 @@
           <t>Spaceplus Perfusor (global catalogue)</t>
         </is>
       </c>
-      <c r="C19" s="32" t="inlineStr">
+      <c r="C19" s="33" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.com/en-01/p/PRID00011858/spaceplus-perfusor</t>
         </is>
@@ -3412,7 +3410,7 @@
           <t>Global website</t>
         </is>
       </c>
-      <c r="E19" s="24" t="inlineStr">
+      <c r="E19" s="28" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -3434,7 +3432,7 @@
           <t>India - Infusion Therapy (navigation)</t>
         </is>
       </c>
-      <c r="C20" s="32" t="inlineStr">
+      <c r="C20" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy</t>
         </is>
@@ -3466,7 +3464,7 @@
           <t>India - Agilia range (lists SP, SP MC, SP TIVA only)</t>
         </is>
       </c>
-      <c r="C21" s="32" t="inlineStr">
+      <c r="C21" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range</t>
         </is>
@@ -3498,7 +3496,7 @@
           <t>India - Infusia range</t>
         </is>
       </c>
-      <c r="C22" s="32" t="inlineStr">
+      <c r="C22" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/infusia-range</t>
         </is>
@@ -3526,7 +3524,7 @@
           <t>Infusia SP7s</t>
         </is>
       </c>
-      <c r="C23" s="32" t="inlineStr">
+      <c r="C23" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/infusia-range/infusia-sp7sed3</t>
         </is>
@@ -3558,7 +3556,7 @@
           <t>Infusia VP7s</t>
         </is>
       </c>
-      <c r="C24" s="32" t="inlineStr">
+      <c r="C24" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/infusia-range/infusia-vp7sed3</t>
         </is>
@@ -3586,7 +3584,7 @@
           <t>Agilia SP</t>
         </is>
       </c>
-      <c r="C25" s="32" t="inlineStr">
+      <c r="C25" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp</t>
         </is>
@@ -3614,7 +3612,7 @@
           <t>Agilia SP MC / SP MC WiFi</t>
         </is>
       </c>
-      <c r="C26" s="32" t="inlineStr">
+      <c r="C26" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp-mc</t>
         </is>
@@ -3646,7 +3644,7 @@
           <t>Agilia SP TIVA</t>
         </is>
       </c>
-      <c r="C27" s="32" t="inlineStr">
+      <c r="C27" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp-tiva</t>
         </is>
@@ -3674,7 +3672,7 @@
           <t>Agilia VP (distributor)</t>
         </is>
       </c>
-      <c r="C28" s="32" t="inlineStr">
+      <c r="C28" s="33" t="inlineStr">
         <is>
           <t>https://arraymed.co.in/product/fresenius-kabi-agilia-vp/</t>
         </is>
@@ -3686,7 +3684,7 @@
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>KEEP (yellow)</t>
+          <t>KEEP (peach)</t>
         </is>
       </c>
       <c r="F28" s="13" t="inlineStr">
@@ -3706,7 +3704,7 @@
           <t>Agilia SP (drug-library evidence)</t>
         </is>
       </c>
-      <c r="C29" s="32" t="inlineStr">
+      <c r="C29" s="33" t="inlineStr">
         <is>
           <t>https://arraymed.co.in/product/fresenius-kabi-agilia-sp/</t>
         </is>
@@ -3718,7 +3716,7 @@
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>ADDED (yellow)</t>
+          <t>ADDED (peach)</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr"/>
@@ -3734,7 +3732,7 @@
           <t>Agilia SP MC (drug-library evidence)</t>
         </is>
       </c>
-      <c r="C30" s="32" t="inlineStr">
+      <c r="C30" s="33" t="inlineStr">
         <is>
           <t>https://arraymed.co.in/product/fresenius-kabi-agilia-spmc/</t>
         </is>
@@ -3746,7 +3744,7 @@
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>ADDED (yellow)</t>
+          <t>ADDED (peach)</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr"/>
@@ -3762,7 +3760,7 @@
           <t>Agilia SP TIVA (WiFi variant evidence)</t>
         </is>
       </c>
-      <c r="C31" s="32" t="inlineStr">
+      <c r="C31" s="33" t="inlineStr">
         <is>
           <t>https://arraymed.co.in/product/fresenius-kabi-agilia-tiva-pump/</t>
         </is>
@@ -3774,7 +3772,7 @@
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>ADDED (yellow)</t>
+          <t>ADDED (peach)</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr"/>
@@ -3790,7 +3788,7 @@
           <t>Agilia SP MC / SP MC WiFi data sheet</t>
         </is>
       </c>
-      <c r="C32" s="32" t="inlineStr">
+      <c r="C32" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/content/dam/fresenius-kabi/gb/products/product-documents/medtech/agilia-connect-sp/IFT265%20Agilia%20SP%20Connect%20Datasheet.pdf.coredownload.inline.pdf</t>
         </is>
@@ -3822,7 +3820,7 @@
           <t>Segment reporting FY2025 (revenue)</t>
         </is>
       </c>
-      <c r="C33" s="32" t="inlineStr">
+      <c r="C33" s="33" t="inlineStr">
         <is>
           <t>https://report.fresenius.com/2025/annual-report/financial-statements/segment-reporting.html</t>
         </is>
@@ -3854,7 +3852,7 @@
           <t>Annual Report 2025 PDF (p.5, p.117)</t>
         </is>
       </c>
-      <c r="C34" s="32" t="inlineStr">
+      <c r="C34" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius.com/sites/default/files/2026-03/fresenius_annual_report_2025_0.pdf</t>
         </is>
@@ -3886,7 +3884,7 @@
           <t>India entity financials</t>
         </is>
       </c>
-      <c r="C35" s="32" t="inlineStr">
+      <c r="C35" s="33" t="inlineStr">
         <is>
           <t>https://www.tofler.in/fresenius-kabi-india-private-limited/company/U24231PN1995PTC014017</t>
         </is>
@@ -3918,7 +3916,7 @@
           <t>GB product literature library</t>
         </is>
       </c>
-      <c r="C36" s="32" t="inlineStr">
+      <c r="C36" s="33" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/gb/healthcare-professional-area/medtech/product-literature-library</t>
         </is>
@@ -3928,7 +3926,7 @@
           <t>Global website (GB HCP area)</t>
         </is>
       </c>
-      <c r="E36" s="24" t="inlineStr">
+      <c r="E36" s="28" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -3950,7 +3948,7 @@
           <t>Key2 Declaration of Conformity</t>
         </is>
       </c>
-      <c r="C37" s="32" t="inlineStr">
+      <c r="C37" s="33" t="inlineStr">
         <is>
           <t>https://key2.fresenius-kabi.com/en/regulatory-document/declaration-conformity/mdr/declaration-conformity</t>
         </is>
@@ -3960,7 +3958,7 @@
           <t>Regulatory document (EU)</t>
         </is>
       </c>
-      <c r="E37" s="24" t="inlineStr">
+      <c r="E37" s="28" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -4060,65 +4058,65 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Method, assumptions and caveats</t>
         </is>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="33" t="inlineStr">
+      <c r="A3" s="34" t="inlineStr">
         <is>
           <t>1. Scope: India market, B. Braun and Fresenius Kabi; syringe and volumetric (large-volume) pumps. BD and Baxter skipped per instruction. Checked October 2026.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="33" t="inlineStr">
-        <is>
-          <t>2. Source priority: (1) company India website, including its catalogue tabs and linked brochures; (2) Indian distributor websites, marked yellow; (3) global company pages/data sheets, used only as backup for features and never as proof of India availability.</t>
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>2. Source priority: (1) company India website, including its catalogue tabs and linked brochures; (2) Indian distributor websites incl. IndiaMart, marked peach; (3) global company pages/data sheets, used only as backup for features and never as proof of India availability.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="33" t="inlineStr">
+      <c r="A5" s="34" t="inlineStr">
         <is>
           <t>3. Visual check: every India page was opened in a real browser and screenshotted (see evidence/ folder). B. Braun catalogue details sit under 'Read more' / 'Overview &amp; Texts' - click there to see drug-library text.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>4. Classification rules applied: an add-on connectivity module (e.g., Data module compactplus) or a separate WiFi variant (e.g., Agilia SP MC vs SP MC WiFi) = 'connectivity optional' = Smart**. A basic RS232 / nurse-call port is NOT counted as connectivity.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="A7" s="34" t="inlineStr">
         <is>
           <t>5. Where a product page is silent on the drug library (e.g., FK Agilia SP, SP TIVA), distributor text was used and the evidence column says so.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="33" t="inlineStr">
-        <is>
-          <t>6. LIMITATION: IndiaMart blocks automated access from this environment (HTTP 429), so the IndiaMart links could not be checked. Agilia VP MC WiFi remains unverified for India.</t>
+      <c r="A8" s="34" t="inlineStr">
+        <is>
+          <t>6. LIMITATION: IndiaMart blocks automated access from this environment (HTTP 429). IndiaMart checks were done manually by the project team; Agilia VP MC WiFi is pending that check.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="A9" s="34" t="inlineStr">
         <is>
           <t>7. LIMITATION: Revenue for the India entities is shown only as ranges (Tofler/Tracxn); exact MCA figures are paywalled. Neither group reports infusion-pump-only revenue; Hospital Care (B. Braun) and MedTech (Fresenius Kabi) are the closest disclosed proxies.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>8. Revenue in USD uses EUR/USD 1.148 (implied by sample) - an editable input on the Revenue tab.</t>
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>8. Revenue in USD uses the latest ECB EUR/USD reference rate 1.1204 (5-Oct-2026) - an editable input on the Revenue tab. Slide shows official (annual report) figures only; India-entity ranges come from aggregators (Tofler/Tracxn) and are kept off the slide. Official India figures would need MCA filings (paid access).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reclassify Agilia VP MC from team-verified IndiaMart listing
IndiaMart lists the base Agilia VP MC (no WiFi variant), so it moves to
Volumetric Smart** (peach); FK Volumetric Connected is now blank.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014jxHyvpwsKVbJ3RxrkkV1k
</commit_message>
<xml_diff>
--- a/Infusion_Pumps_India/Infusion_Pump_Classification_India.xlsx
+++ b/Infusion_Pumps_India/Infusion_Pump_Classification_India.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Product Evidence'!$A$1:$M$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Clean URL Map'!$A$1:$F$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Clean URL Map'!$A$1:$F$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -236,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -270,9 +270,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -295,9 +292,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -307,6 +301,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -861,7 +858,7 @@
       <c r="K6" s="16" t="n"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Pending confirmation of an Indian distributor listing</t>
+          <t>Pending confirmation of an Indian listing (none open)</t>
         </is>
       </c>
     </row>
@@ -944,16 +941,12 @@
           <t>Infusia VP7s (VP7sED3)</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
-        <is>
-          <t>Agilia VP MC WiFi (pending India confirmation)</t>
-        </is>
-      </c>
+      <c r="I9" s="15" t="n"/>
       <c r="J9" s="13" t="inlineStr">
         <is>
           <t>- Add Agilia SP (Smart), Agilia SP MC &amp; SP TIVA (Smart**)
 - Agilia VP (distributor only) -&gt; Volumetric Smart, peach
-- Agilia VP MC WiFi: pending distributor confirmation (keep only if an Indian listing is found)
+- 'Agilia VP MC WiFi' -&gt; India listing (IndiaMart) is base Agilia VP MC -&gt; Volumetric Smart** (peach); Volumetric Connected now blank
 - Infusia SP7s/VP7s &amp; Agilia SP MC WiFi confirmed</t>
         </is>
       </c>
@@ -970,12 +963,12 @@
       </c>
       <c r="F10" s="18" t="n"/>
       <c r="G10" s="17" t="n"/>
-      <c r="H10" s="20" t="inlineStr">
+      <c r="H10" s="19" t="inlineStr">
         <is>
           <t>Agilia VP</t>
         </is>
       </c>
-      <c r="I10" s="18" t="n"/>
+      <c r="I10" s="17" t="n"/>
       <c r="J10" s="17" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
@@ -990,8 +983,12 @@
       </c>
       <c r="F11" s="18" t="n"/>
       <c r="G11" s="17" t="n"/>
-      <c r="H11" s="18" t="n"/>
-      <c r="I11" s="18" t="n"/>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>Agilia VP MC**</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="n"/>
       <c r="J11" s="17" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -1007,25 +1004,25 @@
       <c r="F12" s="18" t="n"/>
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="18" t="n"/>
-      <c r="I12" s="18" t="n"/>
+      <c r="I12" s="10" t="n"/>
       <c r="J12" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>** Smart** = drug library + connectivity optional (separately sold data module / WiFi variant).  * USD converted at ECB EUR/USD reference rate 1.1204 (5-Oct-2026), latest available; sample slide had used ~1.148.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>BD and Baxter excluded from this pass per instruction. Product-level evidence and URLs: see 'Product Evidence' tab.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="J9:J12"/>
     <mergeCell ref="D9:D12"/>
     <mergeCell ref="C9:C12"/>
@@ -1033,6 +1030,7 @@
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="G9:G12"/>
     <mergeCell ref="C6:C8"/>
+    <mergeCell ref="I9:I12"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="J4:J5"/>
     <mergeCell ref="G4:I4"/>
@@ -1143,7 +1141,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>Perfusor compact</t>
         </is>
@@ -1168,12 +1166,12 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="G2" s="22" t="inlineStr">
+      <c r="G2" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H2" s="23" t="inlineStr">
+      <c r="H2" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000461</t>
         </is>
@@ -1210,7 +1208,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>Perfusor compact S</t>
         </is>
@@ -1235,12 +1233,12 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="G3" s="22" t="inlineStr">
+      <c r="G3" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H3" s="23" t="inlineStr">
+      <c r="H3" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000145</t>
         </is>
@@ -1277,7 +1275,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Perfusor compactplus</t>
         </is>
@@ -1302,12 +1300,12 @@
           <t>Smart**</t>
         </is>
       </c>
-      <c r="G4" s="22" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00010216</t>
         </is>
@@ -1340,7 +1338,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Perfusor Space</t>
         </is>
@@ -1365,12 +1363,12 @@
           <t>Smart**</t>
         </is>
       </c>
-      <c r="G5" s="22" t="inlineStr">
+      <c r="G5" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H5" s="23" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00001226</t>
         </is>
@@ -1407,7 +1405,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Spaceplus Perfusor</t>
         </is>
@@ -1432,12 +1430,12 @@
           <t>Excluded - not offered in India</t>
         </is>
       </c>
-      <c r="G6" s="24" t="inlineStr">
+      <c r="G6" s="23" t="inlineStr">
         <is>
           <t>Not offered in India</t>
         </is>
       </c>
-      <c r="H6" s="25" t="inlineStr">
+      <c r="H6" s="24" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00011858 (returns 'No results')</t>
         </is>
@@ -1474,7 +1472,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Infusomat fmS</t>
         </is>
@@ -1499,12 +1497,12 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="G7" s="22" t="inlineStr">
+      <c r="G7" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H7" s="23" t="inlineStr">
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000618</t>
         </is>
@@ -1537,7 +1535,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Infusomat P</t>
         </is>
@@ -1562,12 +1560,12 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="G8" s="22" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H8" s="23" t="inlineStr">
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000689</t>
         </is>
@@ -1600,7 +1598,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Infusomat compactplus</t>
         </is>
@@ -1625,12 +1623,12 @@
           <t>Smart**</t>
         </is>
       </c>
-      <c r="G9" s="22" t="inlineStr">
+      <c r="G9" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H9" s="23" t="inlineStr">
+      <c r="H9" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00011042</t>
         </is>
@@ -1663,7 +1661,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Infusomat compactplus P</t>
         </is>
@@ -1688,12 +1686,12 @@
           <t>Smart**</t>
         </is>
       </c>
-      <c r="G10" s="22" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H10" s="23" t="inlineStr">
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00012086</t>
         </is>
@@ -1730,7 +1728,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Infusomat Space P</t>
         </is>
@@ -1755,12 +1753,12 @@
           <t>Smart**</t>
         </is>
       </c>
-      <c r="G11" s="22" t="inlineStr">
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H11" s="23" t="inlineStr">
+      <c r="H11" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00001230</t>
         </is>
@@ -1793,7 +1791,7 @@
           <t>B. Braun</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Spaceplus Infusomat</t>
         </is>
@@ -1818,12 +1816,12 @@
           <t>Connected</t>
         </is>
       </c>
-      <c r="G12" s="22" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H12" s="23" t="inlineStr">
+      <c r="H12" s="22" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00011860</t>
         </is>
@@ -1856,7 +1854,7 @@
           <t>Fresenius Kabi</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>Infusia SP7s (SP7sED3)</t>
         </is>
@@ -1881,12 +1879,12 @@
           <t>Smart</t>
         </is>
       </c>
-      <c r="G13" s="22" t="inlineStr">
+      <c r="G13" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H13" s="23" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/infusia-range/infusia-sp7sed3</t>
         </is>
@@ -1923,7 +1921,7 @@
           <t>Fresenius Kabi</t>
         </is>
       </c>
-      <c r="B14" s="22" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>Agilia SP</t>
         </is>
@@ -1948,12 +1946,12 @@
           <t>Smart</t>
         </is>
       </c>
-      <c r="G14" s="22" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H14" s="23" t="inlineStr">
+      <c r="H14" s="22" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp</t>
         </is>
@@ -1990,7 +1988,7 @@
           <t>Fresenius Kabi</t>
         </is>
       </c>
-      <c r="B15" s="22" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>Agilia SP MC</t>
         </is>
@@ -2015,12 +2013,12 @@
           <t>Smart**</t>
         </is>
       </c>
-      <c r="G15" s="22" t="inlineStr">
+      <c r="G15" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H15" s="23" t="inlineStr">
+      <c r="H15" s="22" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp-mc</t>
         </is>
@@ -2053,7 +2051,7 @@
           <t>Fresenius Kabi</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>Agilia SP MC WiFi</t>
         </is>
@@ -2078,12 +2076,12 @@
           <t>Connected</t>
         </is>
       </c>
-      <c r="G16" s="22" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H16" s="23" t="inlineStr">
+      <c r="H16" s="22" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp-mc</t>
         </is>
@@ -2120,7 +2118,7 @@
           <t>Fresenius Kabi</t>
         </is>
       </c>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>Agilia SP TIVA</t>
         </is>
@@ -2145,12 +2143,12 @@
           <t>Smart**</t>
         </is>
       </c>
-      <c r="G17" s="22" t="inlineStr">
+      <c r="G17" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H17" s="23" t="inlineStr">
+      <c r="H17" s="22" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp-tiva</t>
         </is>
@@ -2187,7 +2185,7 @@
           <t>Fresenius Kabi</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>Infusia VP7s (VP7sED3)</t>
         </is>
@@ -2212,12 +2210,12 @@
           <t>Smart</t>
         </is>
       </c>
-      <c r="G18" s="22" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
       </c>
-      <c r="H18" s="23" t="inlineStr">
+      <c r="H18" s="22" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/infusia-range/infusia-vp7sed3</t>
         </is>
@@ -2250,7 +2248,7 @@
           <t>Fresenius Kabi</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="25" t="inlineStr">
         <is>
           <t>Agilia VP</t>
         </is>
@@ -2275,12 +2273,12 @@
           <t>Smart</t>
         </is>
       </c>
-      <c r="G19" s="26" t="inlineStr">
+      <c r="G19" s="25" t="inlineStr">
         <is>
           <t>Third-party (India distributor)</t>
         </is>
       </c>
-      <c r="H19" s="27" t="inlineStr">
+      <c r="H19" s="26" t="inlineStr">
         <is>
           <t>https://arraymed.co.in/product/fresenius-kabi-agilia-vp/</t>
         </is>
@@ -2317,9 +2315,9 @@
           <t>Fresenius Kabi</t>
         </is>
       </c>
-      <c r="B20" s="28" t="inlineStr">
-        <is>
-          <t>Agilia VP MC WiFi</t>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>Agilia VP MC</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -2329,52 +2327,52 @@
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>Yes (global) - FK data sheet: 'Up to 19 embedded drug libraries'.</t>
+          <t>Yes - FK data sheet: 'Up to 19 embedded drug libraries'; 'Drug library to be created with Agilia Vigilant Drug'Lib'.</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>Integrated WiFi on WiFi variant (global) - 'Wireless LAN (For Agilia VP MC WiFi only)'.</t>
+          <t>Optional - WiFi only on the separate Agilia VP MC WiFi variant (data sheet: 'Wireless LAN (For Agilia VP MC WiFi only)'). The WiFi variant was not found listed in India.</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Connected (global only)</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="inlineStr">
-        <is>
-          <t>Not verified in India</t>
-        </is>
-      </c>
-      <c r="H20" s="28" t="inlineStr">
-        <is>
-          <t>Pending - not on FK India site or Arraymed; IndiaMart search for team check: https://dir.indiamart.com/search.mp?ss=agilia+vp+mc+wifi</t>
+          <t>Smart**</t>
+        </is>
+      </c>
+      <c r="G20" s="25" t="inlineStr">
+        <is>
+          <t>Third-party (India distributor)</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>https://dir.indiamart.com/search.mp?ss=agilia+vp+mc+wifi (listing: 'Fresenius Kabi Agilia VP MC'; product-page URL to be added)</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>Global data sheet: https://www.fresenius-kabi.com/content/dam/fresenius-kabi/gb/products/product-documents/medtech/agilia-connect-vp/IFT264%20Agilia%20VPMC%20Connect%20Data%20Sheet.pdf.coredownload.inline.pdf</t>
+          <t>FK data sheet p.1-2: https://www.fresenius-kabi.com/content/dam/fresenius-kabi/gb/products/product-documents/medtech/agilia-connect-vp/IFT264%20Agilia%20VPMC%20Connect%20Data%20Sheet.pdf.coredownload.inline.pdf</t>
         </is>
       </c>
       <c r="J20" s="13" t="inlineStr">
         <is>
-          <t>Connected (Indian distributors' websites)</t>
+          <t>Connected - 'Agilia VP MC WiFi' (Indian distributors' websites)</t>
         </is>
       </c>
       <c r="K20" s="13" t="inlineStr">
         <is>
-          <t>PENDING team confirmation of IndiaMart/distributor listing; remove if none</t>
+          <t>RECLASSIFY: India listing is base Agilia VP MC -&gt; Volumetric-Smart**; WiFi variant not listed in India -&gt; FK Volumetric-Connected now blank</t>
         </is>
       </c>
       <c r="L20" s="13" t="inlineStr">
         <is>
-          <t>IndiaMart blocks automated access (HTTP 429), so IndiaMart could not be checked. Manual check needed.</t>
+          <t>IndiaMart listing verified manually by project team (Oct-2026 screenshot); no price shown; seller not captured. Search for 'agilia vp mc wifi' returned no WiFi-variant listing.</t>
         </is>
       </c>
       <c r="M20" s="13" t="inlineStr">
         <is>
-          <t>FK_IN_Agilia_range.jpg (absence)</t>
+          <t>IndiaMart_search_Agilia_VP_MC_team_check.jpg</t>
         </is>
       </c>
     </row>
@@ -2399,6 +2397,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2427,7 +2426,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Revenue cross-check (FY2025)</t>
         </is>
@@ -2439,7 +2438,7 @@
           <t>EUR/USD rate (input)</t>
         </is>
       </c>
-      <c r="B2" s="30" t="n">
+      <c r="B2" s="28" t="n">
         <v>1.1204</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2521,10 +2520,10 @@
           <t>FY2025 (Dec-25)</t>
         </is>
       </c>
-      <c r="D5" s="31" t="n">
+      <c r="D5" s="29" t="n">
         <v>9396</v>
       </c>
-      <c r="E5" s="32">
+      <c r="E5" s="30">
         <f>IF(D5="","n/a",D5*$B$2/1000)</f>
         <v/>
       </c>
@@ -2570,10 +2569,10 @@
           <t>FY2025</t>
         </is>
       </c>
-      <c r="D6" s="31" t="n">
+      <c r="D6" s="29" t="n">
         <v>5090.8</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="30">
         <f>IF(D6="","n/a",D6*$B$2/1000)</f>
         <v/>
       </c>
@@ -2619,8 +2618,8 @@
           <t>FY2025 (Mar-25)</t>
         </is>
       </c>
-      <c r="D7" s="31" t="n"/>
-      <c r="E7" s="32">
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="30">
         <f>IF(D7="","n/a",D7*$B$2/1000)</f>
         <v/>
       </c>
@@ -2666,10 +2665,10 @@
           <t>FY2025 (Dec-25)</t>
         </is>
       </c>
-      <c r="D8" s="31" t="n">
+      <c r="D8" s="29" t="n">
         <v>8612</v>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="30">
         <f>IF(D8="","n/a",D8*$B$2/1000)</f>
         <v/>
       </c>
@@ -2715,10 +2714,10 @@
           <t>FY2025</t>
         </is>
       </c>
-      <c r="D9" s="31" t="n">
+      <c r="D9" s="29" t="n">
         <v>1610</v>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="30">
         <f>IF(D9="","n/a",D9*$B$2/1000)</f>
         <v/>
       </c>
@@ -2764,8 +2763,8 @@
           <t>FY2025 (Mar-25)</t>
         </is>
       </c>
-      <c r="D10" s="31" t="n"/>
-      <c r="E10" s="32">
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="30">
         <f>IF(D10="","n/a",D10*$B$2/1000)</f>
         <v/>
       </c>
@@ -2814,7 +2813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2868,12 +2867,12 @@
           <t>India catalogue - automated infusion systems (master list)</t>
         </is>
       </c>
-      <c r="C2" s="33" t="inlineStr">
+      <c r="C2" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/c/PRODUCTS0000000529/automated-infusion-systems</t>
         </is>
       </c>
-      <c r="D2" s="22" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -2900,12 +2899,12 @@
           <t>Perfusor compact</t>
         </is>
       </c>
-      <c r="C3" s="33" t="inlineStr">
+      <c r="C3" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000461</t>
         </is>
       </c>
-      <c r="D3" s="22" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -2932,12 +2931,12 @@
           <t>Perfusor compact S</t>
         </is>
       </c>
-      <c r="C4" s="33" t="inlineStr">
+      <c r="C4" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000145</t>
         </is>
       </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -2964,12 +2963,12 @@
           <t>Perfusor compactplus</t>
         </is>
       </c>
-      <c r="C5" s="33" t="inlineStr">
+      <c r="C5" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00010216</t>
         </is>
       </c>
-      <c r="D5" s="22" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -2996,12 +2995,12 @@
           <t>Data module compactplus (connectivity add-on)</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00011150</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3028,7 +3027,7 @@
           <t>compactplus brochure (p.5 data module, p.6 DoseGuard)</t>
         </is>
       </c>
-      <c r="C7" s="33" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>https://ecatalog.bbraun.com/eDoc/QlBSMDAwMDAwMDAwMDAwMDAwMTAwMDE4NTA5OTAwMDAw?openInline=true</t>
         </is>
@@ -3056,12 +3055,12 @@
           <t>Perfusor Space</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00001226</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3088,12 +3087,12 @@
           <t>Infusomat fmS</t>
         </is>
       </c>
-      <c r="C9" s="33" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000618</t>
         </is>
       </c>
-      <c r="D9" s="22" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3120,12 +3119,12 @@
           <t>Infusomat P</t>
         </is>
       </c>
-      <c r="C10" s="33" t="inlineStr">
+      <c r="C10" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00000689</t>
         </is>
       </c>
-      <c r="D10" s="22" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3152,12 +3151,12 @@
           <t>Infusomat compactplus</t>
         </is>
       </c>
-      <c r="C11" s="33" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00011042</t>
         </is>
       </c>
-      <c r="D11" s="22" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3184,12 +3183,12 @@
           <t>Infusomat compactplus P</t>
         </is>
       </c>
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C12" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00012086</t>
         </is>
       </c>
-      <c r="D12" s="22" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3212,12 +3211,12 @@
           <t>Infusomat Space P</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00001230</t>
         </is>
       </c>
-      <c r="D13" s="22" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3240,12 +3239,12 @@
           <t>Spaceplus Infusomat</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.co.in/en-IN/p/PRID00011860</t>
         </is>
       </c>
-      <c r="D14" s="22" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3272,7 +3271,7 @@
           <t>Annual Report 2025 (revenue)</t>
         </is>
       </c>
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C15" s="31" t="inlineStr">
         <is>
           <t>https://www.bbraun.com/en/about-us/company/facts-and-figures/annual-report.html</t>
         </is>
@@ -3304,7 +3303,7 @@
           <t>Annual Report 2025 PDF (p.8, p.43)</t>
         </is>
       </c>
-      <c r="C16" s="33" t="inlineStr">
+      <c r="C16" s="31" t="inlineStr">
         <is>
           <t>https://www.bbraun.com/content/dam/b-braun/master/website-6/en/04_about-us/0401_company/facts-and-figures/2025_B_Braun_Annual_Report.pdf</t>
         </is>
@@ -3336,7 +3335,7 @@
           <t>India entity financials</t>
         </is>
       </c>
-      <c r="C17" s="33" t="inlineStr">
+      <c r="C17" s="31" t="inlineStr">
         <is>
           <t>https://www.tofler.in/b-braun-medical-india-private-limited/company/U33112MH1984PTC214514</t>
         </is>
@@ -3368,7 +3367,7 @@
           <t>compactplus system (global page)</t>
         </is>
       </c>
-      <c r="C18" s="33" t="inlineStr">
+      <c r="C18" s="31" t="inlineStr">
         <is>
           <t>https://www.bbraun.com/en/products-and-solutions/therapies/infusion-therapy/automated-infusion-systems/compactplus-system.html</t>
         </is>
@@ -3378,7 +3377,7 @@
           <t>Global website</t>
         </is>
       </c>
-      <c r="E18" s="28" t="inlineStr">
+      <c r="E18" s="32" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -3400,7 +3399,7 @@
           <t>Spaceplus Perfusor (global catalogue)</t>
         </is>
       </c>
-      <c r="C19" s="33" t="inlineStr">
+      <c r="C19" s="31" t="inlineStr">
         <is>
           <t>https://catalogs.bbraun.com/en-01/p/PRID00011858/spaceplus-perfusor</t>
         </is>
@@ -3410,7 +3409,7 @@
           <t>Global website</t>
         </is>
       </c>
-      <c r="E19" s="28" t="inlineStr">
+      <c r="E19" s="32" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -3432,12 +3431,12 @@
           <t>India - Infusion Therapy (navigation)</t>
         </is>
       </c>
-      <c r="C20" s="33" t="inlineStr">
+      <c r="C20" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy</t>
         </is>
       </c>
-      <c r="D20" s="22" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3464,12 +3463,12 @@
           <t>India - Agilia range (lists SP, SP MC, SP TIVA only)</t>
         </is>
       </c>
-      <c r="C21" s="33" t="inlineStr">
+      <c r="C21" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range</t>
         </is>
       </c>
-      <c r="D21" s="22" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3496,12 +3495,12 @@
           <t>India - Infusia range</t>
         </is>
       </c>
-      <c r="C22" s="33" t="inlineStr">
+      <c r="C22" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/infusia-range</t>
         </is>
       </c>
-      <c r="D22" s="22" t="inlineStr">
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3524,12 +3523,12 @@
           <t>Infusia SP7s</t>
         </is>
       </c>
-      <c r="C23" s="33" t="inlineStr">
+      <c r="C23" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/infusia-range/infusia-sp7sed3</t>
         </is>
       </c>
-      <c r="D23" s="22" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3556,12 +3555,12 @@
           <t>Infusia VP7s</t>
         </is>
       </c>
-      <c r="C24" s="33" t="inlineStr">
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/infusia-range/infusia-vp7sed3</t>
         </is>
       </c>
-      <c r="D24" s="22" t="inlineStr">
+      <c r="D24" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3584,12 +3583,12 @@
           <t>Agilia SP</t>
         </is>
       </c>
-      <c r="C25" s="33" t="inlineStr">
+      <c r="C25" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp</t>
         </is>
       </c>
-      <c r="D25" s="22" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3612,12 +3611,12 @@
           <t>Agilia SP MC / SP MC WiFi</t>
         </is>
       </c>
-      <c r="C26" s="33" t="inlineStr">
+      <c r="C26" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp-mc</t>
         </is>
       </c>
-      <c r="D26" s="22" t="inlineStr">
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3644,12 +3643,12 @@
           <t>Agilia SP TIVA</t>
         </is>
       </c>
-      <c r="C27" s="33" t="inlineStr">
+      <c r="C27" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/in/products/ins/infusion-therapy/agilia-range/agilia-sp-tiva</t>
         </is>
       </c>
-      <c r="D27" s="22" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>Official India website</t>
         </is>
@@ -3672,12 +3671,12 @@
           <t>Agilia VP (distributor)</t>
         </is>
       </c>
-      <c r="C28" s="33" t="inlineStr">
+      <c r="C28" s="31" t="inlineStr">
         <is>
           <t>https://arraymed.co.in/product/fresenius-kabi-agilia-vp/</t>
         </is>
       </c>
-      <c r="D28" s="26" t="inlineStr">
+      <c r="D28" s="25" t="inlineStr">
         <is>
           <t>Third-party (India distributor)</t>
         </is>
@@ -3704,12 +3703,12 @@
           <t>Agilia SP (drug-library evidence)</t>
         </is>
       </c>
-      <c r="C29" s="33" t="inlineStr">
+      <c r="C29" s="31" t="inlineStr">
         <is>
           <t>https://arraymed.co.in/product/fresenius-kabi-agilia-sp/</t>
         </is>
       </c>
-      <c r="D29" s="26" t="inlineStr">
+      <c r="D29" s="25" t="inlineStr">
         <is>
           <t>Third-party (India distributor)</t>
         </is>
@@ -3732,12 +3731,12 @@
           <t>Agilia SP MC (drug-library evidence)</t>
         </is>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C30" s="31" t="inlineStr">
         <is>
           <t>https://arraymed.co.in/product/fresenius-kabi-agilia-spmc/</t>
         </is>
       </c>
-      <c r="D30" s="26" t="inlineStr">
+      <c r="D30" s="25" t="inlineStr">
         <is>
           <t>Third-party (India distributor)</t>
         </is>
@@ -3760,12 +3759,12 @@
           <t>Agilia SP TIVA (WiFi variant evidence)</t>
         </is>
       </c>
-      <c r="C31" s="33" t="inlineStr">
+      <c r="C31" s="31" t="inlineStr">
         <is>
           <t>https://arraymed.co.in/product/fresenius-kabi-agilia-tiva-pump/</t>
         </is>
       </c>
-      <c r="D31" s="26" t="inlineStr">
+      <c r="D31" s="25" t="inlineStr">
         <is>
           <t>Third-party (India distributor)</t>
         </is>
@@ -3788,7 +3787,7 @@
           <t>Agilia SP MC / SP MC WiFi data sheet</t>
         </is>
       </c>
-      <c r="C32" s="33" t="inlineStr">
+      <c r="C32" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/content/dam/fresenius-kabi/gb/products/product-documents/medtech/agilia-connect-sp/IFT265%20Agilia%20SP%20Connect%20Datasheet.pdf.coredownload.inline.pdf</t>
         </is>
@@ -3820,7 +3819,7 @@
           <t>Segment reporting FY2025 (revenue)</t>
         </is>
       </c>
-      <c r="C33" s="33" t="inlineStr">
+      <c r="C33" s="31" t="inlineStr">
         <is>
           <t>https://report.fresenius.com/2025/annual-report/financial-statements/segment-reporting.html</t>
         </is>
@@ -3852,7 +3851,7 @@
           <t>Annual Report 2025 PDF (p.5, p.117)</t>
         </is>
       </c>
-      <c r="C34" s="33" t="inlineStr">
+      <c r="C34" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius.com/sites/default/files/2026-03/fresenius_annual_report_2025_0.pdf</t>
         </is>
@@ -3884,7 +3883,7 @@
           <t>India entity financials</t>
         </is>
       </c>
-      <c r="C35" s="33" t="inlineStr">
+      <c r="C35" s="31" t="inlineStr">
         <is>
           <t>https://www.tofler.in/fresenius-kabi-india-private-limited/company/U24231PN1995PTC014017</t>
         </is>
@@ -3916,7 +3915,7 @@
           <t>GB product literature library</t>
         </is>
       </c>
-      <c r="C36" s="33" t="inlineStr">
+      <c r="C36" s="31" t="inlineStr">
         <is>
           <t>https://www.fresenius-kabi.com/gb/healthcare-professional-area/medtech/product-literature-library</t>
         </is>
@@ -3926,7 +3925,7 @@
           <t>Global website (GB HCP area)</t>
         </is>
       </c>
-      <c r="E36" s="28" t="inlineStr">
+      <c r="E36" s="32" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -3948,7 +3947,7 @@
           <t>Key2 Declaration of Conformity</t>
         </is>
       </c>
-      <c r="C37" s="33" t="inlineStr">
+      <c r="C37" s="31" t="inlineStr">
         <is>
           <t>https://key2.fresenius-kabi.com/en/regulatory-document/declaration-conformity/mdr/declaration-conformity</t>
         </is>
@@ -3958,7 +3957,7 @@
           <t>Regulatory document (EU)</t>
         </is>
       </c>
-      <c r="E37" s="28" t="inlineStr">
+      <c r="E37" s="32" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
@@ -3972,37 +3971,101 @@
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
+          <t>Fresenius Kabi</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Agilia VP MC (IndiaMart search; team-verified listing)</t>
+        </is>
+      </c>
+      <c r="C38" s="31" t="inlineStr">
+        <is>
+          <t>https://dir.indiamart.com/search.mp?ss=agilia+vp+mc+wifi</t>
+        </is>
+      </c>
+      <c r="D38" s="25" t="inlineStr">
+        <is>
+          <t>Third-party (India distributor)</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>ADDED (peach)</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>Replace with the product-page URL of the 'Fresenius Kabi Agilia VP MC' listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>Fresenius Kabi</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Agilia VP MC / VP MC WiFi data sheet</t>
+        </is>
+      </c>
+      <c r="C39" s="31" t="inlineStr">
+        <is>
+          <t>https://www.fresenius-kabi.com/content/dam/fresenius-kabi/gb/products/product-documents/medtech/agilia-connect-vp/IFT264%20Agilia%20VPMC%20Connect%20Data%20Sheet.pdf.coredownload.inline.pdf</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Company brochure (global)</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>ADDED (backup)</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>'Wireless LAN (For Agilia VP MC WiFi only)'; 19 drug libraries</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
           <t>BD / Baxter</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>All BD and Baxter URLs</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
+      <c r="C40" s="13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="D40" s="13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="E40" s="13" t="inlineStr">
         <is>
           <t>OUT OF SCOPE</t>
         </is>
       </c>
-      <c r="F38" s="13" t="inlineStr">
+      <c r="F40" s="13" t="inlineStr">
         <is>
           <t>Skipped per instruction</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F38"/>
+  <autoFilter ref="A1:F40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -4040,6 +4103,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4058,63 +4123,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Method, assumptions and caveats</t>
         </is>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="34" t="inlineStr">
+      <c r="A3" s="33" t="inlineStr">
         <is>
           <t>1. Scope: India market, B. Braun and Fresenius Kabi; syringe and volumetric (large-volume) pumps. BD and Baxter skipped per instruction. Checked October 2026.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="34" t="inlineStr">
+      <c r="A4" s="33" t="inlineStr">
         <is>
           <t>2. Source priority: (1) company India website, including its catalogue tabs and linked brochures; (2) Indian distributor websites incl. IndiaMart, marked peach; (3) global company pages/data sheets, used only as backup for features and never as proof of India availability.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="34" t="inlineStr">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t>3. Visual check: every India page was opened in a real browser and screenshotted (see evidence/ folder). B. Braun catalogue details sit under 'Read more' / 'Overview &amp; Texts' - click there to see drug-library text.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="34" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>4. Classification rules applied: an add-on connectivity module (e.g., Data module compactplus) or a separate WiFi variant (e.g., Agilia SP MC vs SP MC WiFi) = 'connectivity optional' = Smart**. A basic RS232 / nurse-call port is NOT counted as connectivity.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="33" t="inlineStr">
         <is>
           <t>5. Where a product page is silent on the drug library (e.g., FK Agilia SP, SP TIVA), distributor text was used and the evidence column says so.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="34" t="inlineStr">
-        <is>
-          <t>6. LIMITATION: IndiaMart blocks automated access from this environment (HTTP 429). IndiaMart checks were done manually by the project team; Agilia VP MC WiFi is pending that check.</t>
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>6. LIMITATION: IndiaMart blocks automated access from this environment (HTTP 429). IndiaMart checks were done manually by the project team (screenshot in evidence/).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="34" t="inlineStr">
+      <c r="A9" s="33" t="inlineStr">
         <is>
           <t>7. LIMITATION: Revenue for the India entities is shown only as ranges (Tofler/Tracxn); exact MCA figures are paywalled. Neither group reports infusion-pump-only revenue; Hospital Care (B. Braun) and MedTech (Fresenius Kabi) are the closest disclosed proxies.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="34" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>8. Revenue in USD uses the latest ECB EUR/USD reference rate 1.1204 (5-Oct-2026) - an editable input on the Revenue tab. Slide shows official (annual report) figures only; India-entity ranges come from aggregators (Tofler/Tracxn) and are kept off the slide. Official India figures would need MCA filings (paid access).</t>
         </is>

</xml_diff>

<commit_message>
Use cleaned IndiaMart search URL (New Delhi) for Agilia VP MC evidence
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014jxHyvpwsKVbJ3RxrkkV1k
</commit_message>
<xml_diff>
--- a/Infusion_Pumps_India/Infusion_Pump_Classification_India.xlsx
+++ b/Infusion_Pumps_India/Infusion_Pump_Classification_India.xlsx
@@ -2347,7 +2347,7 @@
       </c>
       <c r="H20" s="26" t="inlineStr">
         <is>
-          <t>https://dir.indiamart.com/search.mp?ss=agilia+vp+mc+wifi (listing: 'Fresenius Kabi Agilia VP MC'; product-page URL to be added)</t>
+          <t>https://dir.indiamart.com/search.mp?ss=agilia+vp+mc+wifi&amp;cq=New-Delhi (listing: 'Fresenius Kabi Agilia VP MC'; product-page URL to be added)</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="C38" s="31" t="inlineStr">
         <is>
-          <t>https://dir.indiamart.com/search.mp?ss=agilia+vp+mc+wifi</t>
+          <t>https://dir.indiamart.com/search.mp?ss=agilia+vp+mc+wifi&amp;cq=New-Delhi</t>
         </is>
       </c>
       <c r="D38" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Exclude Agilia SP TIVA (specialty TCI/anaesthesia pump) from market scope
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014jxHyvpwsKVbJ3RxrkkV1k
</commit_message>
<xml_diff>
--- a/Infusion_Pumps_India/Infusion_Pump_Classification_India.xlsx
+++ b/Infusion_Pumps_India/Infusion_Pump_Classification_India.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -944,7 +944,8 @@
       <c r="I9" s="15" t="n"/>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>- Add Agilia SP (Smart), Agilia SP MC &amp; SP TIVA (Smart**)
+          <t>- Add Agilia SP (Smart), Agilia SP MC (Smart**)
+- Agilia SP TIVA excluded: specialty TCI/anaesthesia pump
 - Agilia VP (distributor only) -&gt; Volumetric Smart, peach
 - 'Agilia VP MC WiFi' -&gt; India listing (IndiaMart) is base Agilia VP MC -&gt; Volumetric Smart** (peach); Volumetric Connected now blank
 - Infusia SP7s/VP7s &amp; Agilia SP MC WiFi confirmed</t>
@@ -972,71 +973,55 @@
       <c r="J10" s="17" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="17" t="n"/>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
       <c r="E11" s="14" t="inlineStr">
         <is>
           <t>Agilia SP MC**</t>
         </is>
       </c>
       <c r="F11" s="18" t="n"/>
-      <c r="G11" s="17" t="n"/>
+      <c r="G11" s="10" t="n"/>
       <c r="H11" s="19" t="inlineStr">
         <is>
           <t>Agilia VP MC**</t>
         </is>
       </c>
-      <c r="I11" s="17" t="n"/>
-      <c r="J11" s="17" t="n"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Agilia SP TIVA**</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="18" t="n"/>
-      <c r="I12" s="10" t="n"/>
-      <c r="J12" s="10" t="n"/>
+      <c r="I11" s="10" t="n"/>
+      <c r="J11" s="10" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>** Smart** = drug library + connectivity optional (separately sold data module / WiFi variant).  * USD converted at ECB EUR/USD reference rate 1.1204 (5-Oct-2026), latest available; sample slide had used ~1.148.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>** Smart** = drug library + connectivity optional (separately sold data module / WiFi variant).  * USD converted at ECB EUR/USD reference rate 1.1204 (5-Oct-2026), latest available; sample slide had used ~1.148.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
           <t>BD and Baxter excluded from this pass per instruction. Product-level evidence and URLs: see 'Product Evidence' tab.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="J9:J12"/>
-    <mergeCell ref="D9:D12"/>
-    <mergeCell ref="C9:C12"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="B9:B12"/>
-    <mergeCell ref="G9:G12"/>
+    <mergeCell ref="I9:I11"/>
+    <mergeCell ref="J9:J11"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="D9:D11"/>
     <mergeCell ref="C6:C8"/>
-    <mergeCell ref="I9:I12"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="J4:J5"/>
+    <mergeCell ref="A9:A11"/>
     <mergeCell ref="G4:I4"/>
+    <mergeCell ref="B9:B11"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A6:A8"/>
+    <mergeCell ref="C9:C11"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="F6:F8"/>
   </mergeCells>
@@ -2140,7 +2125,7 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Smart**</t>
+          <t>Excluded - specialty TCI/anaesthesia pump</t>
         </is>
       </c>
       <c r="G17" s="21" t="inlineStr">
@@ -2165,12 +2150,12 @@
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
-          <t>ADD to Syringe-Smart**</t>
+          <t>EXCLUDED from market scope (specialty TCI / anaesthesia pump, per project team)</t>
         </is>
       </c>
       <c r="L17" s="13" t="inlineStr">
         <is>
-          <t>Anaesthesia (TCI) niche pump.</t>
+          <t>Would be Smart** on features (drug library; WiFi variant), but sits in the specialty anaesthesia segment, not general infusion.</t>
         </is>
       </c>
       <c r="M17" s="13" t="inlineStr">
@@ -3655,10 +3640,14 @@
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>ADDED</t>
-        </is>
-      </c>
-      <c r="F27" s="13" t="inlineStr"/>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Specialty TCI/anaesthesia pump - out of market scope; keep for reference only</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
@@ -3771,10 +3760,14 @@
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>ADDED (peach)</t>
-        </is>
-      </c>
-      <c r="F31" s="13" t="inlineStr"/>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>Specialty TCI/anaesthesia pump - out of market scope</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
@@ -4132,7 +4125,7 @@
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="33" t="inlineStr">
         <is>
-          <t>1. Scope: India market, B. Braun and Fresenius Kabi; syringe and volumetric (large-volume) pumps. BD and Baxter skipped per instruction. Checked October 2026.</t>
+          <t>1. Scope: India market, B. Braun and Fresenius Kabi; general-purpose syringe and volumetric (large-volume) pumps. Specialty anaesthesia/TCI pumps (e.g., Agilia SP TIVA) excluded. BD and Baxter skipped per instruction. Checked October 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>